<commit_message>
Aug 2 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0041159_VerifiyTheFunctionalityOfVerballyEngagedCFEngagement.xlsx
+++ b/TestData/LV_TMTT0041159_VerifiyTheFunctionalityOfVerballyEngagedCFEngagement.xlsx
@@ -8,18 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D89EA98-3C8B-4AC0-815C-3B009D28B93D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2211DF59-74DA-4332-A6AF-C9AD3E1848C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
-    <sheet name="CAOUsers" sheetId="13" r:id="rId2"/>
-    <sheet name="AppName" sheetId="3" r:id="rId3"/>
-    <sheet name="ModuleName" sheetId="4" r:id="rId4"/>
-    <sheet name="AddOpportunity" sheetId="12" r:id="rId5"/>
-    <sheet name="AddContact" sheetId="14" r:id="rId6"/>
-    <sheet name="VEValidationList" sheetId="15" r:id="rId7"/>
+    <sheet name="AppName" sheetId="3" r:id="rId2"/>
+    <sheet name="ModuleName" sheetId="4" r:id="rId3"/>
+    <sheet name="AddOpportunity" sheetId="12" r:id="rId4"/>
+    <sheet name="AddContact" sheetId="14" r:id="rId5"/>
+    <sheet name="VEValidationList" sheetId="15" r:id="rId6"/>
+    <sheet name="NewOpportunityCounterparty" sheetId="16" r:id="rId7"/>
+    <sheet name="FilterSections" sheetId="17" r:id="rId8"/>
+    <sheet name="CounterpartyContact" sheetId="18" r:id="rId9"/>
+    <sheet name="CounterpartyComments" sheetId="19" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="110">
   <si>
     <t>James Craven</t>
   </si>
@@ -276,6 +279,102 @@
   </si>
   <si>
     <t>System Administrator</t>
+  </si>
+  <si>
+    <t>Engagements</t>
+  </si>
+  <si>
+    <t>Companyname</t>
+  </si>
+  <si>
+    <t>Geller &amp; Company</t>
+  </si>
+  <si>
+    <t>Financial</t>
+  </si>
+  <si>
+    <t>FilterSections</t>
+  </si>
+  <si>
+    <t>SubFilters</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Get Companies from existing Company List</t>
+  </si>
+  <si>
+    <t>Company List</t>
+  </si>
+  <si>
+    <t>2022 Summit Attendees</t>
+  </si>
+  <si>
+    <t>Engagement</t>
+  </si>
+  <si>
+    <t>Swiss Alps</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>Auto-Test Comments</t>
+  </si>
+  <si>
+    <t>ContactName</t>
+  </si>
+  <si>
+    <t>Alan Test</t>
+  </si>
+  <si>
+    <t>FilterType</t>
+  </si>
+  <si>
+    <t>Industry/Product Focus</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>8K Miles</t>
+  </si>
+  <si>
+    <t>FIG</t>
+  </si>
+  <si>
+    <t>Get Companies from existing Engagement</t>
+  </si>
+  <si>
+    <t>CommentsType</t>
+  </si>
+  <si>
+    <t>CommentsText</t>
+  </si>
+  <si>
+    <t>Administrative</t>
+  </si>
+  <si>
+    <t>Internal</t>
+  </si>
+  <si>
+    <t>Next Steps</t>
+  </si>
+  <si>
+    <t>Administrative Comments</t>
+  </si>
+  <si>
+    <t>Internal Comments</t>
+  </si>
+  <si>
+    <t>External Comments</t>
+  </si>
+  <si>
+    <t>Next Steps Comments</t>
   </si>
 </sst>
 </file>
@@ -325,7 +424,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -335,6 +434,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -616,13 +716,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -630,7 +730,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -638,7 +738,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -646,12 +746,66 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>76</v>
       </c>
       <c r="B4" t="s">
         <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68BDA5E3-E591-4217-B969-32786CE2AACB}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -660,20 +814,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FBB8EB1-471A-4668-845A-6810E22F6BA4}">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -682,44 +837,26 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -728,19 +865,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="16.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -835,7 +972,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -937,22 +1074,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>57</v>
       </c>
@@ -978,7 +1115,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>51</v>
       </c>
@@ -1009,22 +1146,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2386AE-B180-4489-BA71-14068DFEFD5A}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="83.140625" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="83.109375" customWidth="1"/>
+    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="96" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>73</v>
       </c>
@@ -1033,4 +1170,140 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1AD5E32-1F75-408B-BF28-CC9346CE869B}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D11B5948-2390-457E-837B-ABA1BE0B3211}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38E383AB-109B-429A-9662-41F16EFC0EA6}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Aug 06 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0041159_VerifiyTheFunctionalityOfVerballyEngagedCFEngagement.xlsx
+++ b/TestData/LV_TMTT0041159_VerifiyTheFunctionalityOfVerballyEngagedCFEngagement.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2211DF59-74DA-4332-A6AF-C9AD3E1848C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30856AC3-3F13-4C4F-A8C3-D73016CBA221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="FilterSections" sheetId="17" r:id="rId8"/>
     <sheet name="CounterpartyContact" sheetId="18" r:id="rId9"/>
     <sheet name="CounterpartyComments" sheetId="19" r:id="rId10"/>
+    <sheet name="EngComments" sheetId="20" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="116">
   <si>
     <t>James Craven</t>
   </si>
@@ -375,6 +376,24 @@
   </si>
   <si>
     <t>Next Steps Comments</t>
+  </si>
+  <si>
+    <t>Kevin Ford</t>
+  </si>
+  <si>
+    <t>Compliance User</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Compliance</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Compliance Comments</t>
+  </si>
+  <si>
+    <t>Compliance</t>
+  </si>
+  <si>
+    <t>Next Step</t>
   </si>
 </sst>
 </file>
@@ -715,14 +734,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -730,7 +749,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -738,7 +757,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -746,12 +765,20 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>76</v>
       </c>
       <c r="B4" t="s">
         <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -761,14 +788,14 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68BDA5E3-E591-4217-B969-32786CE2AACB}">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>101</v>
       </c>
@@ -776,7 +803,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>103</v>
       </c>
@@ -784,7 +811,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>104</v>
       </c>
@@ -792,7 +819,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>66</v>
       </c>
@@ -800,12 +827,20 @@
         <v>108</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>105</v>
       </c>
       <c r="B5" t="s">
         <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -813,22 +848,53 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE4B432-C4FF-4884-91C2-898367FA5347}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+        <v>101</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>103</v>
+      </c>
+      <c r="B2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -836,25 +902,48 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -868,16 +957,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -972,7 +1061,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -1077,19 +1166,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>57</v>
       </c>
@@ -1115,7 +1204,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>51</v>
       </c>
@@ -1149,19 +1238,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2386AE-B180-4489-BA71-14068DFEFD5A}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="83.109375" customWidth="1"/>
-    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="83.140625" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" ht="96" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="96" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>73</v>
       </c>
@@ -1175,13 +1264,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1AD5E32-1F75-408B-BF28-CC9346CE869B}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>79</v>
       </c>
@@ -1192,7 +1281,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>80</v>
       </c>
@@ -1211,14 +1300,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D11B5948-2390-457E-837B-ABA1BE0B3211}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>82</v>
       </c>
@@ -1229,7 +1318,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>100</v>
       </c>
@@ -1240,7 +1329,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>85</v>
       </c>
@@ -1259,13 +1348,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38E383AB-109B-429A-9662-41F16EFC0EA6}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>92</v>
       </c>
@@ -1276,7 +1365,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>93</v>
       </c>
@@ -1287,7 +1376,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>95</v>
       </c>
@@ -1295,7 +1384,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>96</v>
       </c>

</xml_diff>

<commit_message>
1159- changes Aug 22-24
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0041159_VerifiyTheFunctionalityOfVerballyEngagedCFEngagement.xlsx
+++ b/TestData/LV_TMTT0041159_VerifiyTheFunctionalityOfVerballyEngagedCFEngagement.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19C9A2DA-5B06-439F-8504-969D347CAEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F1C0ABF-04DD-4397-B2BB-CC5417533342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="117">
   <si>
     <t>James Craven</t>
   </si>
@@ -1181,10 +1181,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
@@ -1222,7 +1222,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="B2" t="s">
         <v>64</v>
@@ -1236,14 +1236,22 @@
       <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
-        <v>67</v>
-      </c>
       <c r="G2" t="s">
         <v>11</v>
       </c>
-      <c r="H2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>91</v>
+      </c>
+      <c r="B3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TMTI0101398  Changes - 23Aug 24
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0041159_VerifiyTheFunctionalityOfVerballyEngagedCFEngagement.xlsx
+++ b/TestData/LV_TMTT0041159_VerifiyTheFunctionalityOfVerballyEngagedCFEngagement.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F1C0ABF-04DD-4397-B2BB-CC5417533342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B217FC-7A7A-4A3C-89D4-09D07E484C18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="121">
   <si>
     <t>James Craven</t>
   </si>
@@ -361,18 +361,6 @@
     <t>Next Steps</t>
   </si>
   <si>
-    <t>Administrative Comments</t>
-  </si>
-  <si>
-    <t>Internal Comments</t>
-  </si>
-  <si>
-    <t>External Comments</t>
-  </si>
-  <si>
-    <t>Next Steps Comments</t>
-  </si>
-  <si>
     <t>Kevin Ford</t>
   </si>
   <si>
@@ -382,9 +370,6 @@
     <t xml:space="preserve"> Compliance</t>
   </si>
   <si>
-    <t xml:space="preserve"> Compliance Comments</t>
-  </si>
-  <si>
     <t>Compliance</t>
   </si>
   <si>
@@ -398,6 +383,33 @@
   </si>
   <si>
     <t>CSDN-0000006544</t>
+  </si>
+  <si>
+    <t>Administrative Counterparty Comments</t>
+  </si>
+  <si>
+    <t>Internal Counterparty Comments</t>
+  </si>
+  <si>
+    <t>External Counterparty Comments</t>
+  </si>
+  <si>
+    <t>Next Steps Counterparty Comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Compliance Counterparty Comments</t>
+  </si>
+  <si>
+    <t>Administrative Eng Comments</t>
+  </si>
+  <si>
+    <t>Internal Eng Comments</t>
+  </si>
+  <si>
+    <t>Next Steps Eng Comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Compliance Eng Comments</t>
   </si>
 </sst>
 </file>
@@ -782,10 +794,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -799,7 +811,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -815,7 +827,7 @@
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -823,7 +835,7 @@
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -831,7 +843,7 @@
         <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -839,15 +851,15 @@
         <v>103</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B6" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -877,7 +889,7 @@
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -885,23 +897,23 @@
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B5" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -1088,7 +1100,7 @@
         <v>68</v>
       </c>
       <c r="D2" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="E2" t="s">
         <v>41</v>
@@ -1281,13 +1293,13 @@
     </row>
     <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B3" s="4"/>
     </row>
     <row r="4" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>